<commit_message>
Support per-recipient PDF attachments in Mail Merge via an Attachment column
Previously every uploaded PDF was sent to every recipient. Now an
optional "Attachment" column in the Excel file (matched by filename,
comma/semicolon-separated for multiple) lets each recipient get their
own file(s) instead — uploads still happen through the existing
dropzone since a web server can't read a file path off the sender's
own machine. Falls back to the old "send everything to everyone"
behavior when no such column exists.

Adds MailMergeRecipient.attachmentNames so per-recipient attachment
names show up accurately in logs/exports instead of a bare count, and
surfaces missing-filename mismatches in both the composer (before
send, blocking it) and the recipient preview.
</commit_message>
<xml_diff>
--- a/public/samples/mail-merge-template.xlsx
+++ b/public/samples/mail-merge-template.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:G4"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
@@ -405,6 +405,7 @@
     <col min="4" max="4" width="24.83203125" customWidth="1"/>
     <col min="5" max="5" width="24.83203125" customWidth="1"/>
     <col min="6" max="6" width="16.83203125" customWidth="1"/>
+    <col min="7" max="7" width="22.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -426,6 +427,9 @@
       <c r="F1" t="str">
         <v>PDF Password</v>
       </c>
+      <c r="G1" t="str">
+        <v>Attachment</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -446,6 +450,9 @@
       <c r="F2" t="str">
         <v/>
       </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -466,6 +473,9 @@
       <c r="F3" t="str">
         <v/>
       </c>
+      <c r="G3" t="str">
+        <v>john_invoice.pdf</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -486,10 +496,13 @@
       <c r="F4" t="str">
         <v>welcome123</v>
       </c>
+      <c r="G4" t="str">
+        <v>priya_offer.pdf</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>